<commit_message>
checkpointing start of OTA work
</commit_message>
<xml_diff>
--- a/config/modbusmap.xlsx
+++ b/config/modbusmap.xlsx
@@ -2,28 +2,41 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gcb\Dropbox\Projects\DwarfNova\Firmware\FluidManifold\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GlennCB\Dropbox\Projects\DwarfNova\Firmware\FluidManifold\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59730AC8-BD8D-4725-BD3B-E57AECD17F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{997C203B-C8F6-4B29-8758-D4858734F3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="23040" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3708" yWindow="1152" windowWidth="20412" windowHeight="15228" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FluidManifold" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FluidManifold!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FluidManifold!$A$1:$O$58</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="181">
   <si>
     <t>ModbusType</t>
   </si>
@@ -512,6 +525,60 @@
   </si>
   <si>
     <t>Manifold block temperature</t>
+  </si>
+  <si>
+    <t>FWUPDSTART</t>
+  </si>
+  <si>
+    <t>firmware update start for FW update over modbus</t>
+  </si>
+  <si>
+    <t>FWUPDEND</t>
+  </si>
+  <si>
+    <t>firmware update end - set after all firmware sent</t>
+  </si>
+  <si>
+    <t>FWUPDABORT</t>
+  </si>
+  <si>
+    <t>firmware update abort - aborts any update in progress</t>
+  </si>
+  <si>
+    <t>FWSIZE</t>
+  </si>
+  <si>
+    <t>firmware size in bytes</t>
+  </si>
+  <si>
+    <t>FWCHECKSUM</t>
+  </si>
+  <si>
+    <t>firmware checksum CRC</t>
+  </si>
+  <si>
+    <t>firmware data - written repeatedly until transfer complete</t>
+  </si>
+  <si>
+    <t>FWDATA</t>
+  </si>
+  <si>
+    <t>FWUPDSTATE</t>
+  </si>
+  <si>
+    <t>firmware update current state</t>
+  </si>
+  <si>
+    <t>FWUPDERR</t>
+  </si>
+  <si>
+    <t>firmware update error code, zero=no error</t>
+  </si>
+  <si>
+    <t>FWUPDPERCENT</t>
+  </si>
+  <si>
+    <t>firmware update percent download complete</t>
   </si>
 </sst>
 </file>
@@ -538,7 +605,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -578,6 +645,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -646,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -697,6 +770,21 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1011,14 +1099,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
     <col min="4" max="4" width="8.109375" customWidth="1"/>
     <col min="5" max="5" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="49.44140625" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.77734375" customWidth="1"/>
     <col min="13" max="13" width="11.109375" customWidth="1"/>
     <col min="14" max="14" width="12.21875" customWidth="1"/>
@@ -1602,125 +1690,113 @@
       <c r="O16" s="2"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="1">
-        <v>1</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F17" s="1">
-        <v>1</v>
-      </c>
-      <c r="G17" s="1">
-        <v>1</v>
-      </c>
-      <c r="H17" s="1" t="s">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="26">
+        <v>100</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="F17" s="26">
+        <v>1</v>
+      </c>
+      <c r="G17" s="26">
+        <v>1</v>
+      </c>
+      <c r="H17" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="L17" s="2">
-        <v>0</v>
-      </c>
+      <c r="I17" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="J17" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="K17" s="7"/>
+      <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="1">
-        <v>2</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F18" s="1">
-        <v>1</v>
-      </c>
-      <c r="G18" s="1">
-        <v>1</v>
-      </c>
-      <c r="H18" s="1" t="s">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="26">
+        <v>101</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="F18" s="26">
+        <v>1</v>
+      </c>
+      <c r="G18" s="26">
+        <v>1</v>
+      </c>
+      <c r="H18" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K18" s="2">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2">
-        <v>0</v>
-      </c>
+      <c r="I18" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="J18" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="K18" s="7"/>
+      <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="19"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="1">
-        <v>10</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F19" s="1">
-        <v>1</v>
-      </c>
-      <c r="G19" s="1">
-        <v>1</v>
-      </c>
-      <c r="H19" s="1" t="s">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="26">
+        <v>102</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="F19" s="26">
+        <v>1</v>
+      </c>
+      <c r="G19" s="26">
+        <v>1</v>
+      </c>
+      <c r="H19" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K19" s="2">
-        <v>-9</v>
-      </c>
-      <c r="L19" s="2">
-        <v>13</v>
-      </c>
+      <c r="I19" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="J19" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="K19" s="7"/>
+      <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="20"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>55</v>
+      </c>
       <c r="D20" s="1">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F20" s="1">
         <v>1</v>
@@ -1732,159 +1808,165 @@
         <v>19</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K20" s="2">
-        <v>-10</v>
+        <v>21</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="L20" s="2">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>67</v>
-      </c>
+      <c r="A21" s="19"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
       <c r="D21" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="F21" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G21" s="1">
         <v>1</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>70</v>
+        <v>19</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L21" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="K21" s="2">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2">
+        <v>0</v>
+      </c>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
-      <c r="O21" s="2" t="s">
-        <v>72</v>
-      </c>
+      <c r="O21" s="2"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="19"/>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
       <c r="D22" s="1">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="F22" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G22" s="1">
         <v>1</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="K22" s="2">
+        <v>-9</v>
+      </c>
+      <c r="L22" s="2">
+        <v>13</v>
+      </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
       <c r="D23" s="1">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="F23" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G23" s="1">
         <v>1</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="L23" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="K23" s="2">
+        <v>-10</v>
+      </c>
+      <c r="L23" s="2">
+        <v>14</v>
+      </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="19"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
+      <c r="A24" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>67</v>
+      </c>
       <c r="D24" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="F24" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G24" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>80</v>
+      <c r="I24" s="3" t="s">
+        <v>70</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="K24" s="2">
-        <v>0</v>
+        <v>71</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -1892,10 +1974,10 @@
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
       <c r="D25" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="F25" s="1">
         <v>16</v>
@@ -1907,30 +1989,26 @@
         <v>69</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="K25" s="2">
-        <v>1</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
-      <c r="O25" s="2" t="s">
-        <v>85</v>
-      </c>
+      <c r="O25" s="2"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="19"/>
       <c r="B26" s="19"/>
       <c r="C26" s="19"/>
-      <c r="D26" s="9">
-        <v>10</v>
+      <c r="D26" s="1">
+        <v>3</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="F26" s="1">
         <v>16</v>
@@ -1942,58 +2020,52 @@
         <v>69</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K26" s="2">
-        <v>0</v>
-      </c>
-      <c r="L26" s="2">
-        <v>0</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="2" t="s">
-        <v>89</v>
-      </c>
+      <c r="O26" s="2"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="19"/>
       <c r="B27" s="19"/>
       <c r="C27" s="19"/>
-      <c r="D27" s="9">
-        <v>11</v>
+      <c r="D27" s="1">
+        <v>4</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F27" s="1">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G27" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>69</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="K27" s="2">
         <v>0</v>
       </c>
-      <c r="L27" s="2">
-        <v>1</v>
-      </c>
+      <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
@@ -2001,10 +2073,10 @@
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
       <c r="D28" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="F28" s="1">
         <v>16</v>
@@ -2016,65 +2088,67 @@
         <v>69</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>93</v>
+        <v>81</v>
+      </c>
+      <c r="K28" s="2">
+        <v>1</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
       <c r="O28" s="2" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="19"/>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
-      <c r="D29" s="1">
-        <v>13</v>
+      <c r="D29" s="9">
+        <v>10</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="F29" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G29" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="L29" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="K29" s="2">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2">
+        <v>0</v>
+      </c>
       <c r="M29" s="2"/>
-      <c r="N29" s="8"/>
+      <c r="N29" s="2"/>
       <c r="O29" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="19"/>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
-      <c r="D30" s="1">
-        <v>15</v>
+      <c r="D30" s="9">
+        <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F30" s="1">
         <v>16</v>
@@ -2085,53 +2159,57 @@
       <c r="H30" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="I30" s="3" t="s">
-        <v>101</v>
+      <c r="I30" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K30" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="L30" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="K30" s="2">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2">
+        <v>1</v>
+      </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
+      <c r="O30" s="2" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="19"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="1">
+        <v>12</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="1">
         <v>16</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="F31" s="1">
-        <v>32</v>
-      </c>
       <c r="G31" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>104</v>
+        <v>69</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K31" s="3" t="s">
-        <v>105</v>
+      <c r="K31" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
@@ -2139,10 +2217,10 @@
       <c r="B32" s="19"/>
       <c r="C32" s="19"/>
       <c r="D32" s="1">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="F32" s="1">
         <v>32</v>
@@ -2153,47 +2231,49 @@
       <c r="H32" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I32" s="3" t="s">
-        <v>108</v>
+      <c r="I32" s="2" t="s">
+        <v>97</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K32" s="3" t="s">
-        <v>109</v>
+      <c r="K32" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="2" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="19"/>
       <c r="B33" s="19"/>
       <c r="C33" s="19"/>
       <c r="D33" s="1">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="F33" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G33" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
@@ -2205,10 +2285,10 @@
       <c r="B34" s="19"/>
       <c r="C34" s="19"/>
       <c r="D34" s="1">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="F34" s="1">
         <v>32</v>
@@ -2220,34 +2300,30 @@
         <v>96</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="K34" s="3">
-        <v>0</v>
+        <v>71</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="L34" s="2"/>
-      <c r="M34" s="10">
-        <v>5</v>
-      </c>
-      <c r="N34" s="11">
-        <v>-5</v>
-      </c>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
       <c r="O34" s="2" t="s">
-        <v>160</v>
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="20"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="19"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
       <c r="D35" s="1">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F35" s="1">
         <v>32</v>
@@ -2259,56 +2335,46 @@
         <v>96</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="K35" s="3">
-        <v>0</v>
-      </c>
-      <c r="L35" s="2">
-        <v>1</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="L35" s="2"/>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
-      <c r="O35" s="2" t="s">
-        <v>119</v>
-      </c>
+      <c r="O35" s="2"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="B36" s="18">
-        <v>4</v>
-      </c>
-      <c r="C36" s="21" t="s">
-        <v>55</v>
-      </c>
+      <c r="A36" s="19"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
       <c r="D36" s="1">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="F36" s="1">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>122</v>
+        <v>96</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K36" s="2" t="s">
-        <v>123</v>
+      <c r="K36" s="3" t="s">
+        <v>112</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
@@ -2320,179 +2386,180 @@
       <c r="B37" s="19"/>
       <c r="C37" s="19"/>
       <c r="D37" s="1">
+        <v>22</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F37" s="1">
+        <v>32</v>
+      </c>
+      <c r="G37" s="1">
         <v>2</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F37" s="1">
-        <v>16</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
       <c r="H37" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>125</v>
+        <v>96</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>114</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>126</v>
+        <v>115</v>
+      </c>
+      <c r="K37" s="3">
+        <v>0</v>
       </c>
       <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
+      <c r="M37" s="10">
+        <v>5</v>
+      </c>
+      <c r="N37" s="11">
+        <v>-5</v>
+      </c>
+      <c r="O37" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="19"/>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
       <c r="D38" s="1">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F38" s="1">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G38" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>128</v>
+        <v>96</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>117</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="L38" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="K38" s="3">
+        <v>0</v>
+      </c>
+      <c r="L38" s="2">
+        <v>1</v>
+      </c>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
+      <c r="O38" s="2" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="19"/>
       <c r="B39" s="19"/>
       <c r="C39" s="19"/>
-      <c r="D39" s="1">
-        <v>4</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F39" s="1">
-        <v>16</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1</v>
-      </c>
-      <c r="H39" s="1" t="s">
+      <c r="D39" s="26">
+        <v>100</v>
+      </c>
+      <c r="E39" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="F39" s="26">
+        <v>32</v>
+      </c>
+      <c r="G39" s="26">
+        <v>2</v>
+      </c>
+      <c r="H39" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="I39" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>58</v>
-      </c>
+      <c r="I39" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="J39" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="K39" s="3"/>
       <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
-      <c r="N39" s="2"/>
+      <c r="M39" s="24"/>
+      <c r="N39" s="25"/>
       <c r="O39" s="2"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="19"/>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
-      <c r="D40" s="1">
-        <v>5</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F40" s="1">
-        <v>8</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
-      <c r="H40" s="1" t="s">
+      <c r="D40" s="26">
+        <v>102</v>
+      </c>
+      <c r="E40" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="F40" s="26">
+        <v>32</v>
+      </c>
+      <c r="G40" s="26">
+        <v>2</v>
+      </c>
+      <c r="H40" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="I40" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>134</v>
-      </c>
+      <c r="I40" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="K40" s="3"/>
       <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="11"/>
       <c r="O40" s="2"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="19"/>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="9">
-        <v>10</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F41" s="1">
-        <v>16</v>
-      </c>
-      <c r="G41" s="1">
-        <v>1</v>
-      </c>
-      <c r="H41" s="1" t="s">
+      <c r="A41" s="20"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="28">
+        <v>200</v>
+      </c>
+      <c r="E41" s="28" t="s">
+        <v>174</v>
+      </c>
+      <c r="F41" s="28">
+        <v>200</v>
+      </c>
+      <c r="G41" s="28">
+        <v>100</v>
+      </c>
+      <c r="H41" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="I41" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K41" s="2">
-        <v>1</v>
-      </c>
-      <c r="L41" s="2">
-        <v>0</v>
-      </c>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2" t="s">
-        <v>89</v>
+      <c r="I41" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="J41" s="28" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="19"/>
-      <c r="B42" s="19"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="9">
-        <v>11</v>
+      <c r="A42" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B42" s="18">
+        <v>4</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42" s="1">
+        <v>1</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="F42" s="1">
         <v>16</v>
@@ -2504,32 +2571,28 @@
         <v>69</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K42" s="2">
-        <v>1</v>
-      </c>
-      <c r="L42" s="2">
-        <v>1</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L42" s="2"/>
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
-      <c r="O42" s="2" t="s">
-        <v>89</v>
-      </c>
+      <c r="O42" s="2"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="19"/>
       <c r="B43" s="19"/>
       <c r="C43" s="19"/>
       <c r="D43" s="1">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="F43" s="1">
         <v>16</v>
@@ -2538,16 +2601,16 @@
         <v>1</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>139</v>
+        <v>69</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
@@ -2558,252 +2621,551 @@
       <c r="A44" s="19"/>
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
-      <c r="D44" s="9">
-        <v>13</v>
+      <c r="D44" s="1">
+        <v>3</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="F44" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G44" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K44" s="2">
-        <v>0</v>
-      </c>
-      <c r="L44" s="2">
-        <v>0</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="L44" s="2"/>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
-      <c r="O44" s="2" t="s">
-        <v>145</v>
-      </c>
+      <c r="O44" s="2"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="19"/>
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
-      <c r="D45" s="9">
-        <v>15</v>
+      <c r="D45" s="1">
+        <v>4</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="F45" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G45" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="K45" s="2">
-        <v>0</v>
-      </c>
-      <c r="L45" s="2">
-        <v>0</v>
-      </c>
-      <c r="M45" s="14">
-        <v>6</v>
-      </c>
-      <c r="N45" s="14">
-        <v>-5</v>
-      </c>
-      <c r="O45" s="2" t="s">
-        <v>149</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="L45" s="2"/>
+      <c r="M45" s="2"/>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="19"/>
       <c r="B46" s="19"/>
       <c r="C46" s="19"/>
-      <c r="D46" s="9">
-        <v>17</v>
+      <c r="D46" s="1">
+        <v>5</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="F46" s="1">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="G46" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="K46" s="2">
-        <v>0</v>
-      </c>
-      <c r="L46" s="2">
-        <v>0</v>
-      </c>
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="2" t="s">
-        <v>152</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="19"/>
       <c r="B47" s="19"/>
       <c r="C47" s="19"/>
-      <c r="D47" s="1">
-        <v>19</v>
+      <c r="D47" s="9">
+        <v>10</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
       <c r="F47" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G47" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>148</v>
+        <v>88</v>
       </c>
       <c r="K47" s="2">
+        <v>1</v>
+      </c>
+      <c r="L47" s="2">
         <v>0</v>
       </c>
-      <c r="L47" s="2">
-        <v>1</v>
-      </c>
-      <c r="M47" s="8">
-        <v>1000</v>
-      </c>
-      <c r="N47" s="8">
-        <v>0</v>
-      </c>
+      <c r="M47" s="2"/>
+      <c r="N47" s="2"/>
       <c r="O47" s="2" t="s">
-        <v>155</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="19"/>
       <c r="B48" s="19"/>
       <c r="C48" s="19"/>
-      <c r="D48" s="1">
+      <c r="D48" s="9">
+        <v>11</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F48" s="1">
+        <v>16</v>
+      </c>
+      <c r="G48" s="1">
+        <v>1</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="K48" s="2">
+        <v>1</v>
+      </c>
+      <c r="L48" s="2">
+        <v>1</v>
+      </c>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A49" s="19"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="1">
+        <v>12</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F49" s="1">
+        <v>16</v>
+      </c>
+      <c r="G49" s="1">
+        <v>1</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="L49" s="2"/>
+      <c r="M49" s="2"/>
+      <c r="N49" s="2"/>
+      <c r="O49" s="2"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A50" s="19"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="9">
+        <v>13</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F50" s="1">
+        <v>32</v>
+      </c>
+      <c r="G50" s="1">
+        <v>2</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K50" s="2">
+        <v>0</v>
+      </c>
+      <c r="L50" s="2">
+        <v>0</v>
+      </c>
+      <c r="M50" s="2"/>
+      <c r="N50" s="2"/>
+      <c r="O50" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A51" s="19"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="9">
+        <v>15</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F51" s="1">
+        <v>32</v>
+      </c>
+      <c r="G51" s="1">
+        <v>2</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="K51" s="2">
+        <v>0</v>
+      </c>
+      <c r="L51" s="2">
+        <v>0</v>
+      </c>
+      <c r="M51" s="14">
+        <v>6</v>
+      </c>
+      <c r="N51" s="14">
+        <v>-5</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A52" s="19"/>
+      <c r="B52" s="19"/>
+      <c r="C52" s="19"/>
+      <c r="D52" s="9">
+        <v>17</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F52" s="1">
+        <v>32</v>
+      </c>
+      <c r="G52" s="1">
+        <v>2</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="K52" s="2">
+        <v>0</v>
+      </c>
+      <c r="L52" s="2">
+        <v>0</v>
+      </c>
+      <c r="M52" s="8"/>
+      <c r="N52" s="8"/>
+      <c r="O52" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A53" s="19"/>
+      <c r="B53" s="19"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="1">
+        <v>19</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F53" s="1">
+        <v>32</v>
+      </c>
+      <c r="G53" s="1">
+        <v>2</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="K53" s="2">
+        <v>0</v>
+      </c>
+      <c r="L53" s="2">
+        <v>1</v>
+      </c>
+      <c r="M53" s="8">
+        <v>1000</v>
+      </c>
+      <c r="N53" s="8">
+        <v>0</v>
+      </c>
+      <c r="O53" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A54" s="19"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="1">
         <v>21</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E54" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F48" s="1">
+      <c r="F54" s="1">
         <v>32</v>
       </c>
-      <c r="G48" s="1">
+      <c r="G54" s="1">
         <v>2</v>
       </c>
-      <c r="H48" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="I54" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="J48" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K54" s="2">
         <v>0</v>
       </c>
-      <c r="L48" s="2">
+      <c r="L54" s="2">
         <v>2</v>
       </c>
-      <c r="M48" s="8">
+      <c r="M54" s="8">
         <v>104.498</v>
       </c>
-      <c r="N48" s="8">
+      <c r="N54" s="8">
         <v>-122.648</v>
       </c>
-      <c r="O48" s="2" t="s">
+      <c r="O54" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="20"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="1">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A55" s="19"/>
+      <c r="B55" s="19"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="1">
         <v>23</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E55" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="F49" s="1">
+      <c r="F55" s="1">
         <v>32</v>
       </c>
-      <c r="G49" s="1">
+      <c r="G55" s="1">
         <v>2</v>
       </c>
-      <c r="H49" s="1" t="s">
+      <c r="H55" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="I55" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J49" s="1" t="s">
+      <c r="J55" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K55" s="2">
         <v>0</v>
       </c>
-      <c r="L49" s="2">
+      <c r="L55" s="2">
         <v>3</v>
       </c>
-      <c r="M49" s="8">
+      <c r="M55" s="8">
         <v>104.498</v>
       </c>
-      <c r="N49" s="8">
+      <c r="N55" s="8">
         <v>-122.648</v>
       </c>
-      <c r="O49" s="2" t="s">
+      <c r="O55" s="2" t="s">
         <v>158</v>
       </c>
     </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A56" s="19"/>
+      <c r="B56" s="19"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="1">
+        <v>100</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F56" s="1">
+        <v>16</v>
+      </c>
+      <c r="G56" s="1">
+        <v>1</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K56" s="2"/>
+      <c r="L56" s="2"/>
+      <c r="M56" s="8"/>
+      <c r="N56" s="8"/>
+      <c r="O56" s="2"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A57" s="19"/>
+      <c r="B57" s="19"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="1">
+        <v>101</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F57" s="1">
+        <v>16</v>
+      </c>
+      <c r="G57" s="1">
+        <v>1</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="K57" s="2"/>
+      <c r="L57" s="2"/>
+      <c r="M57" s="8"/>
+      <c r="N57" s="8"/>
+      <c r="O57" s="2"/>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A58" s="20"/>
+      <c r="B58" s="20"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="1">
+        <v>102</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F58" s="1">
+        <v>16</v>
+      </c>
+      <c r="G58" s="1">
+        <v>1</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K58" s="2"/>
+      <c r="L58" s="2"/>
+      <c r="M58" s="8"/>
+      <c r="N58" s="8"/>
+      <c r="O58" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O49" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:O58" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="9">
-    <mergeCell ref="A36:A49"/>
-    <mergeCell ref="C36:C49"/>
-    <mergeCell ref="B36:B49"/>
-    <mergeCell ref="A21:A35"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="C21:C35"/>
-    <mergeCell ref="C17:C20"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="B21:B35"/>
+    <mergeCell ref="A42:A58"/>
+    <mergeCell ref="C42:C58"/>
+    <mergeCell ref="B42:B58"/>
+    <mergeCell ref="A24:A41"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="C24:C41"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="B24:B41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Erase standby OTA partition on boot after a successful update (0.17->0.18)
Speeds up the next update by moving the erase cost to boot time (idle)
instead of the update's write loop. Fires once per genuine OTA
switch-over via esp_ota_erase_last_boot_app_partition(), gated on the
same ESP_OTA_IMG_PENDING_VERIFY check as mark_app_valid_cancel_rollback().

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/modbusmap.xlsx
+++ b/config/modbusmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gcb\Dropbox\Projects\DwarfNova\Firmware\FluidManifold\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DAE212B-6C5A-4817-8DF2-43A1E73556AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA1F653-680E-4159-817C-83CC11182C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="23040" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="FluidManifold" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FluidManifold!$A$1:$O$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FluidManifold!$A$1:$O$61</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="191">
   <si>
     <t>ModbusType</t>
   </si>
@@ -572,6 +572,30 @@
   </si>
   <si>
     <t>firmware update - exact bytes written to flash so far (read after a lost/timed-out ack to verify before resending)</t>
+  </si>
+  <si>
+    <t>TESTCOILS</t>
+  </si>
+  <si>
+    <t>scratch coils for link reliability testing</t>
+  </si>
+  <si>
+    <t>TESTCONTS</t>
+  </si>
+  <si>
+    <t>scratch contacts for link reliability testing</t>
+  </si>
+  <si>
+    <t>test holdregs for link reliability testing</t>
+  </si>
+  <si>
+    <t>TESTHREGS</t>
+  </si>
+  <si>
+    <t>TESTIREGS</t>
+  </si>
+  <si>
+    <t>test inregs for link reliability testing</t>
   </si>
 </sst>
 </file>
@@ -712,7 +736,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -756,12 +780,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -792,6 +810,26 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1106,7 +1144,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
@@ -1715,7 +1753,7 @@
       <c r="H17" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="23" t="s">
+      <c r="I17" s="21" t="s">
         <v>55</v>
       </c>
       <c r="J17" s="19" t="s">
@@ -1746,7 +1784,7 @@
       <c r="H18" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="23" t="s">
+      <c r="I18" s="21" t="s">
         <v>57</v>
       </c>
       <c r="J18" s="19" t="s">
@@ -1777,7 +1815,7 @@
       <c r="H19" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="23" t="s">
+      <c r="I19" s="21" t="s">
         <v>59</v>
       </c>
       <c r="J19" s="19" t="s">
@@ -1790,55 +1828,49 @@
       <c r="O19" s="2"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" s="1">
-        <v>1</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="1">
-        <v>1</v>
-      </c>
-      <c r="G20" s="1">
-        <v>1</v>
-      </c>
-      <c r="H20" s="1" t="s">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="38">
+        <v>110</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>183</v>
+      </c>
+      <c r="F20" s="38">
+        <v>10</v>
+      </c>
+      <c r="G20" s="38">
+        <v>10</v>
+      </c>
+      <c r="H20" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L20" s="2">
-        <v>0</v>
-      </c>
+      <c r="I20" s="39" t="s">
+        <v>184</v>
+      </c>
+      <c r="J20" s="40"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="25"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
+      <c r="A21" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>62</v>
+      </c>
       <c r="D21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F21" s="1">
         <v>1</v>
@@ -1850,13 +1882,13 @@
         <v>19</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K21" s="2">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="L21" s="2">
         <v>0</v>
@@ -1866,14 +1898,14 @@
       <c r="O21" s="2"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="25"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
       <c r="D22" s="1">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F22" s="1">
         <v>1</v>
@@ -1885,30 +1917,30 @@
         <v>19</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="2">
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="L22" s="2">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
       <c r="D23" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F23" s="1">
         <v>1</v>
@@ -1920,87 +1952,79 @@
         <v>19</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>31</v>
       </c>
       <c r="K23" s="2">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="L23" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="24" t="s">
-        <v>74</v>
-      </c>
+      <c r="A24" s="23"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
       <c r="D24" s="1">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F24" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G24" s="1">
         <v>1</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>77</v>
+        <v>19</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>71</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L24" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="K24" s="2">
+        <v>-10</v>
+      </c>
+      <c r="L24" s="2">
+        <v>14</v>
+      </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="O24" s="2"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A25" s="25"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
       <c r="D25" s="1">
-        <v>2</v>
+        <v>110</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="F25" s="1">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G25" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>76</v>
+        <v>19</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>82</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="J25" s="1"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -2008,14 +2032,20 @@
       <c r="O25" s="2"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="25"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
+      <c r="A26" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>74</v>
+      </c>
       <c r="D26" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="F26" s="1">
         <v>16</v>
@@ -2026,64 +2056,62 @@
       <c r="H26" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="I26" s="2" t="s">
-        <v>84</v>
+      <c r="I26" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>78</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="O26" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="25"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
+      <c r="A27" s="23"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
       <c r="D27" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F27" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G27" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>76</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K27" s="2">
-        <v>0</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="K27" s="2"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
-      <c r="O27" s="2" t="s">
-        <v>89</v>
-      </c>
+      <c r="O27" s="2"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="25"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
+      <c r="A28" s="23"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
       <c r="D28" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F28" s="1">
         <v>16</v>
@@ -2095,67 +2123,63 @@
         <v>76</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K28" s="2">
-        <v>1</v>
+        <v>78</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
-      <c r="O28" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="O28" s="2"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="9">
-        <v>10</v>
+      <c r="A29" s="23"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="1">
+        <v>4</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F29" s="1">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G29" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>76</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="K29" s="2">
         <v>0</v>
       </c>
-      <c r="L29" s="2">
-        <v>0</v>
-      </c>
+      <c r="L29" s="2"/>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="25"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="9">
-        <v>11</v>
+      <c r="A30" s="23"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="1">
+        <v>6</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="F30" s="1">
         <v>16</v>
@@ -2167,32 +2191,30 @@
         <v>76</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="K30" s="2">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L30" s="2"/>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="25"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="1">
-        <v>12</v>
+      <c r="A31" s="23"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="9">
+        <v>10</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="F31" s="1">
         <v>16</v>
@@ -2204,65 +2226,69 @@
         <v>76</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="L31" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="K31" s="2">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2">
+        <v>0</v>
+      </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="25"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="1">
-        <v>13</v>
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="9">
+        <v>11</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F32" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G32" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="L32" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="K32" s="2">
+        <v>0</v>
+      </c>
+      <c r="L32" s="2">
+        <v>1</v>
+      </c>
       <c r="M32" s="2"/>
-      <c r="N32" s="8"/>
+      <c r="N32" s="2"/>
       <c r="O32" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="25"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
+      <c r="A33" s="23"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
       <c r="D33" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="F33" s="1">
         <v>16</v>
@@ -2273,29 +2299,31 @@
       <c r="H33" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="I33" s="3" t="s">
-        <v>108</v>
+      <c r="I33" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="K33" s="3" t="s">
-        <v>109</v>
+      <c r="K33" s="2" t="s">
+        <v>100</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
+      <c r="O33" s="2" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="25"/>
-      <c r="B34" s="25"/>
-      <c r="C34" s="25"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
       <c r="D34" s="1">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="F34" s="1">
         <v>32</v>
@@ -2306,49 +2334,49 @@
       <c r="H34" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="I34" s="3" t="s">
-        <v>111</v>
+      <c r="I34" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="K34" s="3" t="s">
-        <v>112</v>
+      <c r="K34" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
+      <c r="N34" s="8"/>
       <c r="O34" s="2" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="25"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
+      <c r="A35" s="23"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
       <c r="D35" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="F35" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G35" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>78</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
@@ -2356,14 +2384,14 @@
       <c r="O35" s="2"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="25"/>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
       <c r="D36" s="1">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="F36" s="1">
         <v>32</v>
@@ -2375,28 +2403,30 @@
         <v>103</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>78</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
+      <c r="O36" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="25"/>
-      <c r="B37" s="25"/>
-      <c r="C37" s="25"/>
+      <c r="A37" s="23"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
       <c r="D37" s="1">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F37" s="1">
         <v>32</v>
@@ -2408,34 +2438,28 @@
         <v>103</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="K37" s="3">
-        <v>0</v>
+        <v>78</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>116</v>
       </c>
       <c r="L37" s="2"/>
-      <c r="M37" s="10">
-        <v>5</v>
-      </c>
-      <c r="N37" s="11">
-        <v>-5</v>
-      </c>
-      <c r="O37" s="2" t="s">
-        <v>123</v>
-      </c>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="25"/>
-      <c r="B38" s="25"/>
-      <c r="C38" s="25"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
       <c r="D38" s="1">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F38" s="1">
         <v>32</v>
@@ -2447,224 +2471,231 @@
         <v>103</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="K38" s="3">
-        <v>0</v>
-      </c>
-      <c r="L38" s="2">
-        <v>1</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="L38" s="2"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
-      <c r="O38" s="2" t="s">
+      <c r="O38" s="2"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A39" s="23"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="1">
+        <v>22</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F39" s="1">
+        <v>32</v>
+      </c>
+      <c r="G39" s="1">
+        <v>2</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="K39" s="3">
+        <v>0</v>
+      </c>
+      <c r="L39" s="2"/>
+      <c r="M39" s="10">
+        <v>5</v>
+      </c>
+      <c r="N39" s="11">
+        <v>-5</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="1">
+        <v>24</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="1">
+        <v>32</v>
+      </c>
+      <c r="G40" s="1">
+        <v>2</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="K40" s="3">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2">
+        <v>1</v>
+      </c>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="25"/>
-      <c r="B39" s="25"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="19">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A41" s="23"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="19">
         <v>100</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E41" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="F39" s="19">
+      <c r="F41" s="19">
         <v>32</v>
       </c>
-      <c r="G39" s="19">
+      <c r="G41" s="19">
         <v>2</v>
       </c>
-      <c r="H39" s="19" t="s">
+      <c r="H41" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="I39" s="20" t="s">
+      <c r="I41" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="J39" s="19" t="s">
+      <c r="J41" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="K39" s="3"/>
-      <c r="L39" s="2"/>
-      <c r="N39" s="18"/>
-      <c r="O39" s="2"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="25"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="19">
+      <c r="K41" s="3"/>
+      <c r="L41" s="2"/>
+      <c r="N41" s="18"/>
+      <c r="O41" s="2"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A42" s="23"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="33">
         <v>102</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E42" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="F40" s="19">
+      <c r="F42" s="33">
         <v>32</v>
       </c>
-      <c r="G40" s="19">
+      <c r="G42" s="33">
         <v>2</v>
       </c>
-      <c r="H40" s="19" t="s">
+      <c r="H42" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="I40" s="20" t="s">
+      <c r="I42" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="J40" s="19" t="s">
+      <c r="J42" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="K40" s="3"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="11"/>
-      <c r="O40" s="2"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="26"/>
-      <c r="B41" s="26"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="21">
+      <c r="K42" s="35"/>
+      <c r="L42" s="18"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="11"/>
+      <c r="O42" s="18"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A43" s="23"/>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="36">
+        <v>110</v>
+      </c>
+      <c r="E43" s="36" t="s">
+        <v>188</v>
+      </c>
+      <c r="F43" s="36">
+        <v>160</v>
+      </c>
+      <c r="G43" s="36">
+        <v>10</v>
+      </c>
+      <c r="H43" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="I43" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="J43" s="36"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="2"/>
+      <c r="M43" s="8"/>
+      <c r="N43" s="8"/>
+      <c r="O43" s="2"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A44" s="24"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="19">
         <v>200</v>
       </c>
-      <c r="E41" s="21" t="s">
+      <c r="E44" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F41" s="21">
+      <c r="F44" s="19">
         <v>1600</v>
       </c>
-      <c r="G41" s="21">
+      <c r="G44" s="19">
         <v>100</v>
       </c>
-      <c r="H41" s="21" t="s">
+      <c r="H44" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="I41" s="22" t="s">
+      <c r="I44" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="J41" s="21" t="s">
+      <c r="J44" s="19" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="B42" s="29">
-        <v>4</v>
-      </c>
-      <c r="C42" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="D42" s="1">
-        <v>1</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F42" s="1">
-        <v>16</v>
-      </c>
-      <c r="G42" s="1">
-        <v>1</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="30"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="1">
-        <v>2</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="F43" s="1">
-        <v>16</v>
-      </c>
-      <c r="G43" s="1">
-        <v>1</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="30"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="33"/>
-      <c r="D44" s="1">
-        <v>3</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="F44" s="1">
-        <v>16</v>
-      </c>
-      <c r="G44" s="1">
-        <v>1</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>143</v>
-      </c>
+      <c r="K44" s="2"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A45" s="30"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="33"/>
+      <c r="A45" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="B45" s="27">
+        <v>4</v>
+      </c>
+      <c r="C45" s="30" t="s">
+        <v>62</v>
+      </c>
       <c r="D45" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="F45" s="1">
         <v>16</v>
@@ -2676,13 +2707,13 @@
         <v>76</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="J45" s="1" t="s">
         <v>78</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>65</v>
+        <v>137</v>
       </c>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
@@ -2690,17 +2721,17 @@
       <c r="O45" s="2"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="30"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="33"/>
+      <c r="A46" s="28"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="31"/>
       <c r="D46" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="F46" s="1">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G46" s="1">
         <v>1</v>
@@ -2709,13 +2740,13 @@
         <v>76</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="J46" s="1" t="s">
         <v>78</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
@@ -2723,14 +2754,14 @@
       <c r="O46" s="2"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A47" s="30"/>
-      <c r="B47" s="30"/>
-      <c r="C47" s="33"/>
-      <c r="D47" s="9">
-        <v>10</v>
+      <c r="A47" s="28"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="1">
+        <v>3</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="F47" s="1">
         <v>16</v>
@@ -2742,32 +2773,28 @@
         <v>76</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="K47" s="2">
-        <v>1</v>
-      </c>
-      <c r="L47" s="2">
-        <v>0</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="L47" s="2"/>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
-      <c r="O47" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="O47" s="2"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A48" s="30"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="33"/>
-      <c r="D48" s="9">
-        <v>11</v>
+      <c r="A48" s="28"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="1">
+        <v>4</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="F48" s="1">
         <v>16</v>
@@ -2779,50 +2806,46 @@
         <v>76</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="K48" s="2">
-        <v>1</v>
-      </c>
-      <c r="L48" s="2">
-        <v>1</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L48" s="2"/>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
-      <c r="O48" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="O48" s="2"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="30"/>
-      <c r="B49" s="30"/>
-      <c r="C49" s="33"/>
+      <c r="A49" s="28"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="31"/>
       <c r="D49" s="1">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F49" s="1">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G49" s="1">
         <v>1</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>153</v>
+        <v>76</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="J49" s="1" t="s">
         <v>78</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="2"/>
@@ -2830,32 +2853,32 @@
       <c r="O49" s="2"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A50" s="30"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="33"/>
+      <c r="A50" s="28"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="31"/>
       <c r="D50" s="9">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F50" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G50" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>158</v>
+        <v>95</v>
       </c>
       <c r="K50" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" s="2">
         <v>0</v>
@@ -2863,96 +2886,88 @@
       <c r="M50" s="2"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2" t="s">
-        <v>159</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A51" s="30"/>
-      <c r="B51" s="30"/>
-      <c r="C51" s="33"/>
+      <c r="A51" s="28"/>
+      <c r="B51" s="28"/>
+      <c r="C51" s="31"/>
       <c r="D51" s="9">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F51" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G51" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>162</v>
+        <v>95</v>
       </c>
       <c r="K51" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2">
-        <v>0</v>
-      </c>
-      <c r="M51" s="14">
-        <v>6</v>
-      </c>
-      <c r="N51" s="14">
-        <v>-5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M51" s="2"/>
+      <c r="N51" s="2"/>
       <c r="O51" s="2" t="s">
-        <v>163</v>
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A52" s="30"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="33"/>
-      <c r="D52" s="9">
-        <v>17</v>
+      <c r="A52" s="28"/>
+      <c r="B52" s="28"/>
+      <c r="C52" s="31"/>
+      <c r="D52" s="1">
+        <v>12</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="F52" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G52" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>103</v>
+        <v>153</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="K52" s="2">
-        <v>0</v>
-      </c>
-      <c r="L52" s="2">
-        <v>0</v>
-      </c>
-      <c r="M52" s="8"/>
-      <c r="N52" s="8"/>
-      <c r="O52" s="2" t="s">
-        <v>166</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+      <c r="O52" s="2"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A53" s="30"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="33"/>
-      <c r="D53" s="1">
-        <v>19</v>
+      <c r="A53" s="28"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="9">
+        <v>13</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="F53" s="1">
         <v>32</v>
@@ -2964,36 +2979,32 @@
         <v>103</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="K53" s="2">
         <v>0</v>
       </c>
       <c r="L53" s="2">
-        <v>1</v>
-      </c>
-      <c r="M53" s="8">
-        <v>1000</v>
-      </c>
-      <c r="N53" s="8">
         <v>0</v>
       </c>
+      <c r="M53" s="2"/>
+      <c r="N53" s="2"/>
       <c r="O53" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A54" s="30"/>
-      <c r="B54" s="30"/>
-      <c r="C54" s="33"/>
-      <c r="D54" s="1">
-        <v>21</v>
+      <c r="A54" s="28"/>
+      <c r="B54" s="28"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="9">
+        <v>15</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="F54" s="1">
         <v>32</v>
@@ -3005,7 +3016,7 @@
         <v>103</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>162</v>
@@ -3014,27 +3025,27 @@
         <v>0</v>
       </c>
       <c r="L54" s="2">
-        <v>2</v>
-      </c>
-      <c r="M54" s="8">
-        <v>104.498</v>
-      </c>
-      <c r="N54" s="8">
-        <v>-122.648</v>
+        <v>0</v>
+      </c>
+      <c r="M54" s="14">
+        <v>6</v>
+      </c>
+      <c r="N54" s="14">
+        <v>-5</v>
       </c>
       <c r="O54" s="2" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A55" s="30"/>
-      <c r="B55" s="30"/>
-      <c r="C55" s="33"/>
-      <c r="D55" s="1">
-        <v>23</v>
+      <c r="A55" s="28"/>
+      <c r="B55" s="28"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="9">
+        <v>17</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="F55" s="1">
         <v>32</v>
@@ -3046,144 +3057,170 @@
         <v>103</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
       <c r="K55" s="2">
         <v>0</v>
       </c>
       <c r="L55" s="2">
+        <v>0</v>
+      </c>
+      <c r="M55" s="8"/>
+      <c r="N55" s="8"/>
+      <c r="O55" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A56" s="28"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="31"/>
+      <c r="D56" s="1">
+        <v>19</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F56" s="1">
+        <v>32</v>
+      </c>
+      <c r="G56" s="1">
+        <v>2</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K56" s="2">
+        <v>0</v>
+      </c>
+      <c r="L56" s="2">
+        <v>1</v>
+      </c>
+      <c r="M56" s="8">
+        <v>1000</v>
+      </c>
+      <c r="N56" s="8">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A57" s="28"/>
+      <c r="B57" s="28"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="1">
+        <v>21</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F57" s="1">
+        <v>32</v>
+      </c>
+      <c r="G57" s="1">
+        <v>2</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K57" s="2">
+        <v>0</v>
+      </c>
+      <c r="L57" s="2">
+        <v>2</v>
+      </c>
+      <c r="M57" s="8">
+        <v>104.498</v>
+      </c>
+      <c r="N57" s="8">
+        <v>-122.648</v>
+      </c>
+      <c r="O57" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A58" s="28"/>
+      <c r="B58" s="28"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="1">
+        <v>23</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F58" s="1">
+        <v>32</v>
+      </c>
+      <c r="G58" s="1">
+        <v>2</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K58" s="2">
+        <v>0</v>
+      </c>
+      <c r="L58" s="2">
         <v>3</v>
       </c>
-      <c r="M55" s="8">
+      <c r="M58" s="8">
         <v>104.498</v>
       </c>
-      <c r="N55" s="8">
+      <c r="N58" s="8">
         <v>-122.648</v>
       </c>
-      <c r="O55" s="2" t="s">
+      <c r="O58" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A56" s="30"/>
-      <c r="B56" s="30"/>
-      <c r="C56" s="33"/>
-      <c r="D56" s="1">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A59" s="28"/>
+      <c r="B59" s="28"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="1">
         <v>100</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E59" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F56" s="1">
+      <c r="F59" s="1">
         <v>16</v>
       </c>
-      <c r="G56" s="1">
-        <v>1</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="K56" s="2"/>
-      <c r="L56" s="2"/>
-      <c r="M56" s="8"/>
-      <c r="N56" s="8"/>
-      <c r="O56" s="2"/>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A57" s="30"/>
-      <c r="B57" s="30"/>
-      <c r="C57" s="33"/>
-      <c r="D57" s="1">
-        <v>101</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="F57" s="1">
-        <v>16</v>
-      </c>
-      <c r="G57" s="1">
-        <v>1</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I57" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="8"/>
-      <c r="N57" s="8"/>
-      <c r="O57" s="2"/>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A58" s="30"/>
-      <c r="B58" s="30"/>
-      <c r="C58" s="33"/>
-      <c r="D58" s="1">
-        <v>102</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F58" s="1">
-        <v>16</v>
-      </c>
-      <c r="G58" s="1">
-        <v>1</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="K58" s="2"/>
-      <c r="L58" s="2"/>
-      <c r="M58" s="8"/>
-      <c r="N58" s="8"/>
-      <c r="O58" s="2"/>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A59" s="31"/>
-      <c r="B59" s="31"/>
-      <c r="C59" s="34"/>
-      <c r="D59" s="1">
-        <v>103</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="F59" s="1">
-        <v>32</v>
-      </c>
       <c r="G59" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H59" s="1" t="s">
         <v>76</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="K59" s="2"/>
       <c r="L59" s="2"/>
@@ -3191,18 +3228,140 @@
       <c r="N59" s="8"/>
       <c r="O59" s="2"/>
     </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A60" s="28"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="31"/>
+      <c r="D60" s="1">
+        <v>101</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F60" s="1">
+        <v>16</v>
+      </c>
+      <c r="G60" s="1">
+        <v>1</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="K60" s="2"/>
+      <c r="L60" s="2"/>
+      <c r="M60" s="8"/>
+      <c r="N60" s="8"/>
+      <c r="O60" s="2"/>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A61" s="28"/>
+      <c r="B61" s="28"/>
+      <c r="C61" s="31"/>
+      <c r="D61" s="1">
+        <v>102</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F61" s="1">
+        <v>16</v>
+      </c>
+      <c r="G61" s="1">
+        <v>1</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K61" s="2"/>
+      <c r="L61" s="2"/>
+      <c r="M61" s="8"/>
+      <c r="N61" s="8"/>
+      <c r="O61" s="2"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A62" s="28"/>
+      <c r="B62" s="28"/>
+      <c r="C62" s="31"/>
+      <c r="D62" s="1">
+        <v>103</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F62" s="1">
+        <v>32</v>
+      </c>
+      <c r="G62" s="1">
+        <v>2</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="K62" s="2"/>
+      <c r="L62" s="2"/>
+      <c r="M62" s="8"/>
+      <c r="N62" s="8"/>
+      <c r="O62" s="2"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A63" s="29"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="32"/>
+      <c r="D63" s="1">
+        <v>110</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F63" s="1">
+        <v>160</v>
+      </c>
+      <c r="G63" s="1">
+        <v>10</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="J63" s="1"/>
+      <c r="K63" s="2"/>
+      <c r="L63" s="2"/>
+      <c r="M63" s="8"/>
+      <c r="N63" s="8"/>
+      <c r="O63" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O58" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:O61" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="9">
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A24:A41"/>
-    <mergeCell ref="C24:C41"/>
-    <mergeCell ref="B24:B41"/>
-    <mergeCell ref="A42:A59"/>
-    <mergeCell ref="B42:B59"/>
-    <mergeCell ref="C42:C59"/>
+    <mergeCell ref="A45:A63"/>
+    <mergeCell ref="B45:B63"/>
+    <mergeCell ref="C45:C63"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="C21:C25"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="A26:A44"/>
+    <mergeCell ref="C26:C44"/>
+    <mergeCell ref="B26:B44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>